<commit_message>
Remove now unused soc by lc transitions table
</commit_message>
<xml_diff>
--- a/te_algorithms/data/summary_table_ld_sdg.xlsx
+++ b/te_algorithms/data/summary_table_ld_sdg.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-26.04\home\azvoleff\Code\LandDegradation\trends.earth-algorithms\te_algorithms\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36AC8682-6E17-44C1-9821-AF320EEA501E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3251D70C-8223-45A5-BB8B-12CE3F5B6775}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SDG 15.3.1" sheetId="5" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="68">
   <si>
     <t>Land area with improved productivity:</t>
   </si>
@@ -226,9 +226,6 @@
   </si>
   <si>
     <t>* Trends.Earth calculates soil organic carbon change based on annual land cover transitions. This table shows change in soil organic carbon based on the initial and final years only. The final year soil organic carbon value used to produce this table accounts for all land cover transitions that ocurred between the initial and final years. An empty cell indicates that transition was not observed over the time period.</t>
-  </si>
-  <si>
-    <t>Soil organic carbon change from initial year to final year by type of land cover transition (as percentage of initial stock)*</t>
   </si>
   <si>
     <t>Percent change in soil organic carbon storage from initial year to final year:</t>
@@ -402,18 +399,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -482,7 +473,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="17">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -491,15 +482,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color auto="1"/>
       </left>
@@ -676,24 +658,6 @@
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -703,15 +667,15 @@
     <xf numFmtId="43" fontId="8" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="86">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -721,7 +685,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -738,34 +702,31 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="4" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -774,7 +735,7 @@
     <xf numFmtId="4" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="7" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -783,17 +744,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="7" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -818,7 +776,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -827,150 +785,129 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="7" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="9" fillId="7" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="9" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="9" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="9" fillId="9" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="13" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="9" fillId="13" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="12" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="9" fillId="12" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="8" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="3" fontId="9" fillId="7" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="12" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="3" fontId="9" fillId="8" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="9" fillId="13" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="9" fillId="9" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1304,10 +1241,10 @@
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="14.5703125" customWidth="1"/>
-    <col min="3" max="5" width="15.5703125" style="34" customWidth="1"/>
-    <col min="6" max="6" width="16.85546875" style="34" customWidth="1"/>
-    <col min="7" max="9" width="15.5703125" style="34" customWidth="1"/>
-    <col min="10" max="10" width="15.5703125" style="35" customWidth="1"/>
+    <col min="3" max="5" width="15.5703125" style="32" customWidth="1"/>
+    <col min="6" max="6" width="16.85546875" style="32" customWidth="1"/>
+    <col min="7" max="9" width="15.5703125" style="32" customWidth="1"/>
+    <col min="10" max="10" width="15.5703125" style="33" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1328,88 +1265,88 @@
       <c r="A2" s="4"/>
     </row>
     <row r="3" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="87" t="s">
+      <c r="A3" s="76" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="87"/>
-      <c r="C3" s="87"/>
-      <c r="D3" s="87"/>
-      <c r="E3" s="87"/>
-      <c r="F3" s="87"/>
-      <c r="G3" s="87"/>
-      <c r="H3" s="87"/>
-      <c r="I3" s="87"/>
-      <c r="J3" s="87"/>
-    </row>
-    <row r="4" spans="1:10" s="36" customFormat="1" ht="30.75" x14ac:dyDescent="0.3">
-      <c r="A4" s="38"/>
-      <c r="C4" s="39"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="39"/>
-      <c r="F4" s="43" t="s">
+      <c r="B3" s="76"/>
+      <c r="C3" s="76"/>
+      <c r="D3" s="76"/>
+      <c r="E3" s="76"/>
+      <c r="F3" s="76"/>
+      <c r="G3" s="76"/>
+      <c r="H3" s="76"/>
+      <c r="I3" s="76"/>
+      <c r="J3" s="76"/>
+    </row>
+    <row r="4" spans="1:10" s="34" customFormat="1" ht="30.75" x14ac:dyDescent="0.3">
+      <c r="A4" s="36"/>
+      <c r="C4" s="37"/>
+      <c r="D4" s="37"/>
+      <c r="E4" s="37"/>
+      <c r="F4" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="G4" s="43" t="s">
+      <c r="G4" s="41" t="s">
         <v>38</v>
       </c>
-      <c r="H4" s="39"/>
-      <c r="I4" s="39"/>
-      <c r="J4" s="40"/>
+      <c r="H4" s="37"/>
+      <c r="I4" s="37"/>
+      <c r="J4" s="38"/>
     </row>
     <row r="5" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
-      <c r="E5" s="28" t="s">
+      <c r="E5" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="F5" s="41">
+      <c r="F5" s="39">
         <f>SUM(F6:F9)</f>
         <v>0</v>
       </c>
-      <c r="G5" s="44" t="e">
+      <c r="G5" s="42" t="e">
         <f>SUM(G6:G9)</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
-      <c r="E6" s="28" t="s">
+      <c r="E6" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="F6" s="45"/>
-      <c r="G6" s="46" t="e">
+      <c r="F6" s="43"/>
+      <c r="G6" s="44" t="e">
         <f>F6/$F$5</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
-      <c r="E7" s="28" t="s">
+      <c r="E7" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="42"/>
-      <c r="G7" s="29" t="e">
+      <c r="F7" s="40"/>
+      <c r="G7" s="28" t="e">
         <f t="shared" ref="G7:G9" si="0">F7/$F$5</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
-      <c r="E8" s="28" t="s">
+      <c r="E8" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="F8" s="49"/>
-      <c r="G8" s="50" t="e">
+      <c r="F8" s="47"/>
+      <c r="G8" s="48" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
-      <c r="E9" s="28" t="s">
+      <c r="E9" s="27" t="s">
         <v>22</v>
       </c>
-      <c r="F9" s="47"/>
-      <c r="G9" s="48" t="e">
+      <c r="F9" s="45"/>
+      <c r="G9" s="46" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
@@ -1417,22 +1354,22 @@
     <row r="10" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
     </row>
-    <row r="11" spans="1:10" s="36" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="88" t="s">
+    <row r="11" spans="1:10" s="34" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="80" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="88"/>
-      <c r="C11" s="88"/>
-      <c r="D11" s="88"/>
-      <c r="E11" s="88"/>
-      <c r="F11" s="88"/>
-      <c r="G11" s="88"/>
-      <c r="H11" s="88"/>
-      <c r="I11" s="88"/>
-      <c r="J11" s="88"/>
+      <c r="B11" s="80"/>
+      <c r="C11" s="80"/>
+      <c r="D11" s="80"/>
+      <c r="E11" s="80"/>
+      <c r="F11" s="80"/>
+      <c r="G11" s="80"/>
+      <c r="H11" s="80"/>
+      <c r="I11" s="80"/>
+      <c r="J11" s="80"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="33" t="s">
+      <c r="A13" s="31" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1453,8 +1390,8 @@
   <cols>
     <col min="1" max="1" width="8.7109375" customWidth="1"/>
     <col min="2" max="2" width="14.5703125" customWidth="1"/>
-    <col min="3" max="9" width="15.5703125" style="34" customWidth="1"/>
-    <col min="10" max="10" width="15.5703125" style="35" customWidth="1"/>
+    <col min="3" max="9" width="15.5703125" style="32" customWidth="1"/>
+    <col min="10" max="10" width="15.5703125" style="33" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -1482,82 +1419,82 @@
       <c r="J2"/>
     </row>
     <row r="3" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="87" t="s">
+      <c r="A3" s="76" t="s">
         <v>46</v>
       </c>
-      <c r="B3" s="89"/>
-      <c r="C3" s="89"/>
-      <c r="D3" s="89"/>
-      <c r="E3" s="89"/>
-      <c r="F3" s="89"/>
-      <c r="G3" s="89"/>
-      <c r="H3" s="89"/>
-      <c r="I3" s="89"/>
-      <c r="J3" s="89"/>
+      <c r="B3" s="77"/>
+      <c r="C3" s="77"/>
+      <c r="D3" s="77"/>
+      <c r="E3" s="77"/>
+      <c r="F3" s="77"/>
+      <c r="G3" s="77"/>
+      <c r="H3" s="77"/>
+      <c r="I3" s="77"/>
+      <c r="J3" s="77"/>
     </row>
     <row r="4" spans="1:10" ht="30.75" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
-      <c r="F4" s="43" t="s">
+      <c r="F4" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="G4" s="43" t="s">
+      <c r="G4" s="41" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
-      <c r="E5" s="28" t="s">
+      <c r="E5" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="F5" s="41">
+      <c r="F5" s="39">
         <f>SUM(F6:F9)</f>
         <v>0</v>
       </c>
-      <c r="G5" s="44" t="e">
+      <c r="G5" s="42" t="e">
         <f>SUM(G6:G9)</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
-      <c r="E6" s="28" t="s">
-        <v>0</v>
-      </c>
-      <c r="F6" s="45"/>
-      <c r="G6" s="46" t="e">
+      <c r="E6" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="F6" s="43"/>
+      <c r="G6" s="44" t="e">
         <f>F6/$F$5</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
-      <c r="E7" s="28" t="s">
+      <c r="E7" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="F7" s="42"/>
-      <c r="G7" s="29" t="e">
+      <c r="F7" s="40"/>
+      <c r="G7" s="28" t="e">
         <f t="shared" ref="G7:G9" si="0">F7/$F$5</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
-      <c r="E8" s="28" t="s">
+      <c r="E8" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="F8" s="49"/>
-      <c r="G8" s="50" t="e">
+      <c r="F8" s="47"/>
+      <c r="G8" s="48" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
-      <c r="E9" s="28" t="s">
+      <c r="E9" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="F9" s="47"/>
-      <c r="G9" s="48" t="e">
+      <c r="F9" s="45"/>
+      <c r="G9" s="46" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
@@ -1566,45 +1503,45 @@
       <c r="A10" s="4"/>
     </row>
     <row r="11" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="88" t="s">
-        <v>68</v>
-      </c>
-      <c r="B11" s="89"/>
-      <c r="C11" s="90"/>
-      <c r="D11" s="90"/>
-      <c r="E11" s="90"/>
-      <c r="F11" s="90"/>
-      <c r="G11" s="90"/>
-      <c r="H11" s="90"/>
-      <c r="I11" s="90"/>
-      <c r="J11" s="91"/>
+      <c r="A11" s="80" t="s">
+        <v>67</v>
+      </c>
+      <c r="B11" s="77"/>
+      <c r="C11" s="81"/>
+      <c r="D11" s="81"/>
+      <c r="E11" s="81"/>
+      <c r="F11" s="81"/>
+      <c r="G11" s="81"/>
+      <c r="H11" s="81"/>
+      <c r="I11" s="81"/>
+      <c r="J11" s="82"/>
     </row>
     <row r="12" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4"/>
     </row>
-    <row r="13" spans="1:10" s="34" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="72" t="s">
+    <row r="13" spans="1:10" s="32" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="68" t="s">
         <v>43</v>
       </c>
-      <c r="B13" s="72"/>
-      <c r="C13" s="72"/>
-      <c r="D13" s="72"/>
-      <c r="E13" s="72"/>
-      <c r="F13" s="72"/>
-      <c r="G13" s="72"/>
-      <c r="H13" s="72"/>
-      <c r="I13" s="72"/>
-      <c r="J13" s="72"/>
-    </row>
-    <row r="14" spans="1:10" s="34" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="68"/>
+      <c r="C13" s="68"/>
+      <c r="D13" s="68"/>
+      <c r="E13" s="68"/>
+      <c r="F13" s="68"/>
+      <c r="G13" s="68"/>
+      <c r="H13" s="68"/>
+      <c r="I13" s="68"/>
+      <c r="J13" s="68"/>
+    </row>
+    <row r="14" spans="1:10" s="32" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="1"/>
-      <c r="C14" s="58" t="s">
+      <c r="C14" s="54" t="s">
         <v>62</v>
       </c>
-      <c r="J14" s="35"/>
+      <c r="J14" s="33"/>
     </row>
     <row r="15" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="C15" s="54" t="s">
+      <c r="C15" s="52" t="s">
         <v>16</v>
       </c>
       <c r="D15" s="14" t="s">
@@ -1625,25 +1562,25 @@
       <c r="I15" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="J15" s="35" t="s">
+      <c r="J15" s="33" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="55" t="s">
+      <c r="A16" s="53" t="s">
         <v>56</v>
       </c>
-      <c r="B16" s="51" t="s">
+      <c r="B16" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="23"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="23"/>
-      <c r="G16" s="23"/>
-      <c r="H16" s="23"/>
-      <c r="I16" s="23"/>
-      <c r="J16" s="25">
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="22"/>
+      <c r="I16" s="22"/>
+      <c r="J16" s="24">
         <f>SUM(C16:I16)</f>
         <v>0</v>
       </c>
@@ -1652,14 +1589,14 @@
       <c r="B17" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C17" s="23"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="23"/>
-      <c r="F17" s="23"/>
-      <c r="G17" s="23"/>
-      <c r="H17" s="23"/>
-      <c r="I17" s="23"/>
-      <c r="J17" s="25">
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="22"/>
+      <c r="F17" s="22"/>
+      <c r="G17" s="22"/>
+      <c r="H17" s="22"/>
+      <c r="I17" s="22"/>
+      <c r="J17" s="24">
         <f t="shared" ref="J17:J22" si="1">SUM(C17:I17)</f>
         <v>0</v>
       </c>
@@ -1668,14 +1605,14 @@
       <c r="B18" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C18" s="23"/>
-      <c r="D18" s="23"/>
-      <c r="E18" s="23"/>
-      <c r="F18" s="23"/>
-      <c r="G18" s="23"/>
-      <c r="H18" s="23"/>
-      <c r="I18" s="23"/>
-      <c r="J18" s="25">
+      <c r="C18" s="22"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="22"/>
+      <c r="H18" s="22"/>
+      <c r="I18" s="22"/>
+      <c r="J18" s="24">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1684,14 +1621,14 @@
       <c r="B19" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C19" s="23"/>
-      <c r="D19" s="23"/>
-      <c r="E19" s="23"/>
-      <c r="F19" s="23"/>
-      <c r="G19" s="23"/>
-      <c r="H19" s="23"/>
-      <c r="I19" s="23"/>
-      <c r="J19" s="25">
+      <c r="C19" s="22"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="22"/>
+      <c r="F19" s="22"/>
+      <c r="G19" s="22"/>
+      <c r="H19" s="22"/>
+      <c r="I19" s="22"/>
+      <c r="J19" s="24">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1700,14 +1637,14 @@
       <c r="B20" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="23"/>
-      <c r="D20" s="23"/>
-      <c r="E20" s="23"/>
-      <c r="F20" s="23"/>
-      <c r="G20" s="23"/>
-      <c r="H20" s="23"/>
-      <c r="I20" s="23"/>
-      <c r="J20" s="25">
+      <c r="C20" s="22"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="22"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="22"/>
+      <c r="I20" s="22"/>
+      <c r="J20" s="24">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1716,14 +1653,14 @@
       <c r="B21" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C21" s="23"/>
-      <c r="D21" s="23"/>
-      <c r="E21" s="23"/>
-      <c r="F21" s="23"/>
-      <c r="G21" s="23"/>
-      <c r="H21" s="23"/>
-      <c r="I21" s="23"/>
-      <c r="J21" s="25">
+      <c r="C21" s="22"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="22"/>
+      <c r="F21" s="22"/>
+      <c r="G21" s="22"/>
+      <c r="H21" s="22"/>
+      <c r="I21" s="22"/>
+      <c r="J21" s="24">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1732,14 +1669,14 @@
       <c r="B22" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C22" s="23"/>
-      <c r="D22" s="23"/>
-      <c r="E22" s="23"/>
-      <c r="F22" s="23"/>
-      <c r="G22" s="23"/>
-      <c r="H22" s="23"/>
-      <c r="I22" s="23"/>
-      <c r="J22" s="25">
+      <c r="C22" s="22"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="22"/>
+      <c r="F22" s="22"/>
+      <c r="G22" s="22"/>
+      <c r="H22" s="22"/>
+      <c r="I22" s="22"/>
+      <c r="J22" s="24">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
@@ -1749,61 +1686,61 @@
       <c r="B23" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C23" s="25">
+      <c r="C23" s="24">
         <f>SUM(C16:C22)</f>
         <v>0</v>
       </c>
-      <c r="D23" s="25">
+      <c r="D23" s="24">
         <f t="shared" ref="D23:J23" si="2">SUM(D16:D22)</f>
         <v>0</v>
       </c>
-      <c r="E23" s="25">
+      <c r="E23" s="24">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="F23" s="25">
+      <c r="F23" s="24">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="G23" s="25">
+      <c r="G23" s="24">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="H23" s="25">
+      <c r="H23" s="24">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="I23" s="25">
+      <c r="I23" s="24">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="J23" s="24">
+      <c r="J23" s="23">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:10" s="34" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="71" t="s">
+    <row r="25" spans="1:10" s="32" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="67" t="s">
         <v>42</v>
       </c>
-      <c r="B25" s="71"/>
-      <c r="C25" s="71"/>
-      <c r="D25" s="71"/>
-      <c r="E25" s="71"/>
-      <c r="F25" s="71"/>
-      <c r="G25" s="71"/>
-      <c r="H25" s="71"/>
-      <c r="I25" s="71"/>
-      <c r="J25" s="71"/>
-    </row>
-    <row r="26" spans="1:10" s="34" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C26" s="58" t="s">
+      <c r="B25" s="67"/>
+      <c r="C25" s="67"/>
+      <c r="D25" s="67"/>
+      <c r="E25" s="67"/>
+      <c r="F25" s="67"/>
+      <c r="G25" s="67"/>
+      <c r="H25" s="67"/>
+      <c r="I25" s="67"/>
+      <c r="J25" s="67"/>
+    </row>
+    <row r="26" spans="1:10" s="32" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C26" s="54" t="s">
         <v>62</v>
       </c>
-      <c r="J26" s="35"/>
+      <c r="J26" s="33"/>
     </row>
     <row r="27" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="C27" s="53" t="s">
+      <c r="C27" s="51" t="s">
         <v>16</v>
       </c>
       <c r="D27" s="3" t="s">
@@ -1824,25 +1761,25 @@
       <c r="I27" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="J27" s="35" t="s">
+      <c r="J27" s="33" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="55" t="s">
+      <c r="A28" s="53" t="s">
         <v>56</v>
       </c>
-      <c r="B28" s="51" t="s">
+      <c r="B28" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="C28" s="23"/>
-      <c r="D28" s="23"/>
-      <c r="E28" s="23"/>
-      <c r="F28" s="23"/>
-      <c r="G28" s="23"/>
-      <c r="H28" s="23"/>
-      <c r="I28" s="23"/>
-      <c r="J28" s="25">
+      <c r="C28" s="22"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="22"/>
+      <c r="F28" s="22"/>
+      <c r="G28" s="22"/>
+      <c r="H28" s="22"/>
+      <c r="I28" s="22"/>
+      <c r="J28" s="24">
         <f>SUM(C28:I28)</f>
         <v>0</v>
       </c>
@@ -1851,14 +1788,14 @@
       <c r="B29" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C29" s="23"/>
-      <c r="D29" s="23"/>
-      <c r="E29" s="23"/>
-      <c r="F29" s="23"/>
-      <c r="G29" s="23"/>
-      <c r="H29" s="23"/>
-      <c r="I29" s="23"/>
-      <c r="J29" s="25">
+      <c r="C29" s="22"/>
+      <c r="D29" s="22"/>
+      <c r="E29" s="22"/>
+      <c r="F29" s="22"/>
+      <c r="G29" s="22"/>
+      <c r="H29" s="22"/>
+      <c r="I29" s="22"/>
+      <c r="J29" s="24">
         <f t="shared" ref="J29:J34" si="3">SUM(C29:I29)</f>
         <v>0</v>
       </c>
@@ -1867,14 +1804,14 @@
       <c r="B30" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C30" s="23"/>
-      <c r="D30" s="23"/>
-      <c r="E30" s="23"/>
-      <c r="F30" s="23"/>
-      <c r="G30" s="23"/>
-      <c r="H30" s="23"/>
-      <c r="I30" s="23"/>
-      <c r="J30" s="25">
+      <c r="C30" s="22"/>
+      <c r="D30" s="22"/>
+      <c r="E30" s="22"/>
+      <c r="F30" s="22"/>
+      <c r="G30" s="22"/>
+      <c r="H30" s="22"/>
+      <c r="I30" s="22"/>
+      <c r="J30" s="24">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -1883,14 +1820,14 @@
       <c r="B31" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C31" s="23"/>
-      <c r="D31" s="23"/>
-      <c r="E31" s="23"/>
-      <c r="F31" s="23"/>
-      <c r="G31" s="23"/>
-      <c r="H31" s="23"/>
-      <c r="I31" s="23"/>
-      <c r="J31" s="25">
+      <c r="C31" s="22"/>
+      <c r="D31" s="22"/>
+      <c r="E31" s="22"/>
+      <c r="F31" s="22"/>
+      <c r="G31" s="22"/>
+      <c r="H31" s="22"/>
+      <c r="I31" s="22"/>
+      <c r="J31" s="24">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -1899,14 +1836,14 @@
       <c r="B32" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C32" s="23"/>
-      <c r="D32" s="23"/>
-      <c r="E32" s="23"/>
-      <c r="F32" s="23"/>
-      <c r="G32" s="23"/>
-      <c r="H32" s="23"/>
-      <c r="I32" s="23"/>
-      <c r="J32" s="25">
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="22"/>
+      <c r="H32" s="22"/>
+      <c r="I32" s="22"/>
+      <c r="J32" s="24">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -1915,14 +1852,14 @@
       <c r="B33" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C33" s="23"/>
-      <c r="D33" s="23"/>
-      <c r="E33" s="23"/>
-      <c r="F33" s="23"/>
-      <c r="G33" s="23"/>
-      <c r="H33" s="23"/>
-      <c r="I33" s="23"/>
-      <c r="J33" s="25">
+      <c r="C33" s="22"/>
+      <c r="D33" s="22"/>
+      <c r="E33" s="22"/>
+      <c r="F33" s="22"/>
+      <c r="G33" s="22"/>
+      <c r="H33" s="22"/>
+      <c r="I33" s="22"/>
+      <c r="J33" s="24">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -1931,14 +1868,14 @@
       <c r="B34" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C34" s="23"/>
-      <c r="D34" s="23"/>
-      <c r="E34" s="23"/>
-      <c r="F34" s="23"/>
-      <c r="G34" s="23"/>
-      <c r="H34" s="23"/>
-      <c r="I34" s="23"/>
-      <c r="J34" s="25">
+      <c r="C34" s="22"/>
+      <c r="D34" s="22"/>
+      <c r="E34" s="22"/>
+      <c r="F34" s="22"/>
+      <c r="G34" s="22"/>
+      <c r="H34" s="22"/>
+      <c r="I34" s="22"/>
+      <c r="J34" s="24">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
@@ -1948,65 +1885,65 @@
       <c r="B35" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C35" s="25">
+      <c r="C35" s="24">
         <f>SUM(C28:C34)</f>
         <v>0</v>
       </c>
-      <c r="D35" s="25">
+      <c r="D35" s="24">
         <f t="shared" ref="D35:J35" si="4">SUM(D28:D34)</f>
         <v>0</v>
       </c>
-      <c r="E35" s="25">
+      <c r="E35" s="24">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="F35" s="25">
+      <c r="F35" s="24">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="G35" s="25">
+      <c r="G35" s="24">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="H35" s="25">
+      <c r="H35" s="24">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="I35" s="25">
+      <c r="I35" s="24">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="J35" s="24">
+      <c r="J35" s="23">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:10" s="34" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="68" t="s">
+    <row r="37" spans="1:10" s="32" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="64" t="s">
         <v>41</v>
       </c>
-      <c r="B37" s="69"/>
-      <c r="C37" s="69"/>
-      <c r="D37" s="69"/>
-      <c r="E37" s="69"/>
-      <c r="F37" s="69"/>
-      <c r="G37" s="69"/>
-      <c r="H37" s="69"/>
-      <c r="I37" s="69"/>
-      <c r="J37" s="70"/>
-    </row>
-    <row r="38" spans="1:10" s="34" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B37" s="65"/>
+      <c r="C37" s="65"/>
+      <c r="D37" s="65"/>
+      <c r="E37" s="65"/>
+      <c r="F37" s="65"/>
+      <c r="G37" s="65"/>
+      <c r="H37" s="65"/>
+      <c r="I37" s="65"/>
+      <c r="J37" s="66"/>
+    </row>
+    <row r="38" spans="1:10" s="32" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="1"/>
-      <c r="C38" s="58" t="s">
+      <c r="C38" s="54" t="s">
         <v>62</v>
       </c>
-      <c r="J38" s="35"/>
+      <c r="J38" s="33"/>
     </row>
     <row r="39" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>67</v>
-      </c>
-      <c r="C39" s="53" t="s">
+        <v>66</v>
+      </c>
+      <c r="C39" s="51" t="s">
         <v>16</v>
       </c>
       <c r="D39" s="3" t="s">
@@ -2027,25 +1964,25 @@
       <c r="I39" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="J39" s="35" t="s">
+      <c r="J39" s="33" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="40" spans="1:10" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="55" t="s">
+      <c r="A40" s="53" t="s">
         <v>56</v>
       </c>
-      <c r="B40" s="51" t="s">
+      <c r="B40" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="C40" s="23"/>
-      <c r="D40" s="23"/>
-      <c r="E40" s="23"/>
-      <c r="F40" s="23"/>
-      <c r="G40" s="23"/>
-      <c r="H40" s="23"/>
-      <c r="I40" s="23"/>
-      <c r="J40" s="25">
+      <c r="C40" s="22"/>
+      <c r="D40" s="22"/>
+      <c r="E40" s="22"/>
+      <c r="F40" s="22"/>
+      <c r="G40" s="22"/>
+      <c r="H40" s="22"/>
+      <c r="I40" s="22"/>
+      <c r="J40" s="24">
         <f>SUM(C40:I40)</f>
         <v>0</v>
       </c>
@@ -2054,14 +1991,14 @@
       <c r="B41" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C41" s="23"/>
-      <c r="D41" s="23"/>
-      <c r="E41" s="23"/>
-      <c r="F41" s="23"/>
-      <c r="G41" s="23"/>
-      <c r="H41" s="23"/>
-      <c r="I41" s="23"/>
-      <c r="J41" s="25">
+      <c r="C41" s="22"/>
+      <c r="D41" s="22"/>
+      <c r="E41" s="22"/>
+      <c r="F41" s="22"/>
+      <c r="G41" s="22"/>
+      <c r="H41" s="22"/>
+      <c r="I41" s="22"/>
+      <c r="J41" s="24">
         <f t="shared" ref="J41:J46" si="5">SUM(C41:I41)</f>
         <v>0</v>
       </c>
@@ -2070,14 +2007,14 @@
       <c r="B42" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C42" s="23"/>
-      <c r="D42" s="23"/>
-      <c r="E42" s="23"/>
-      <c r="F42" s="23"/>
-      <c r="G42" s="23"/>
-      <c r="H42" s="23"/>
-      <c r="I42" s="23"/>
-      <c r="J42" s="25">
+      <c r="C42" s="22"/>
+      <c r="D42" s="22"/>
+      <c r="E42" s="22"/>
+      <c r="F42" s="22"/>
+      <c r="G42" s="22"/>
+      <c r="H42" s="22"/>
+      <c r="I42" s="22"/>
+      <c r="J42" s="24">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -2086,14 +2023,14 @@
       <c r="B43" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C43" s="23"/>
-      <c r="D43" s="23"/>
-      <c r="E43" s="23"/>
-      <c r="F43" s="23"/>
-      <c r="G43" s="23"/>
-      <c r="H43" s="23"/>
-      <c r="I43" s="23"/>
-      <c r="J43" s="25">
+      <c r="C43" s="22"/>
+      <c r="D43" s="22"/>
+      <c r="E43" s="22"/>
+      <c r="F43" s="22"/>
+      <c r="G43" s="22"/>
+      <c r="H43" s="22"/>
+      <c r="I43" s="22"/>
+      <c r="J43" s="24">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -2102,14 +2039,14 @@
       <c r="B44" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C44" s="23"/>
-      <c r="D44" s="23"/>
-      <c r="E44" s="23"/>
-      <c r="F44" s="23"/>
-      <c r="G44" s="23"/>
-      <c r="H44" s="23"/>
-      <c r="I44" s="23"/>
-      <c r="J44" s="25">
+      <c r="C44" s="22"/>
+      <c r="D44" s="22"/>
+      <c r="E44" s="22"/>
+      <c r="F44" s="22"/>
+      <c r="G44" s="22"/>
+      <c r="H44" s="22"/>
+      <c r="I44" s="22"/>
+      <c r="J44" s="24">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -2118,14 +2055,14 @@
       <c r="B45" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C45" s="23"/>
-      <c r="D45" s="23"/>
-      <c r="E45" s="23"/>
-      <c r="F45" s="23"/>
-      <c r="G45" s="23"/>
-      <c r="H45" s="23"/>
-      <c r="I45" s="23"/>
-      <c r="J45" s="25">
+      <c r="C45" s="22"/>
+      <c r="D45" s="22"/>
+      <c r="E45" s="22"/>
+      <c r="F45" s="22"/>
+      <c r="G45" s="22"/>
+      <c r="H45" s="22"/>
+      <c r="I45" s="22"/>
+      <c r="J45" s="24">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -2134,14 +2071,14 @@
       <c r="B46" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C46" s="23"/>
-      <c r="D46" s="23"/>
-      <c r="E46" s="23"/>
-      <c r="F46" s="23"/>
-      <c r="G46" s="23"/>
-      <c r="H46" s="23"/>
-      <c r="I46" s="23"/>
-      <c r="J46" s="25">
+      <c r="C46" s="22"/>
+      <c r="D46" s="22"/>
+      <c r="E46" s="22"/>
+      <c r="F46" s="22"/>
+      <c r="G46" s="22"/>
+      <c r="H46" s="22"/>
+      <c r="I46" s="22"/>
+      <c r="J46" s="24">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -2151,62 +2088,62 @@
       <c r="B47" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C47" s="25">
+      <c r="C47" s="24">
         <f>SUM(C40:C46)</f>
         <v>0</v>
       </c>
-      <c r="D47" s="25">
+      <c r="D47" s="24">
         <f t="shared" ref="D47:J47" si="6">SUM(D40:D46)</f>
         <v>0</v>
       </c>
-      <c r="E47" s="25">
+      <c r="E47" s="24">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="F47" s="25">
+      <c r="F47" s="24">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G47" s="25">
+      <c r="G47" s="24">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="H47" s="25">
+      <c r="H47" s="24">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="I47" s="25">
+      <c r="I47" s="24">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="J47" s="24">
+      <c r="J47" s="23">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:10" s="34" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="65" t="s">
+    <row r="49" spans="1:10" s="32" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="61" t="s">
         <v>44</v>
       </c>
-      <c r="B49" s="66"/>
-      <c r="C49" s="66"/>
-      <c r="D49" s="66"/>
-      <c r="E49" s="66"/>
-      <c r="F49" s="66"/>
-      <c r="G49" s="66"/>
-      <c r="H49" s="66"/>
-      <c r="I49" s="66"/>
-      <c r="J49" s="67"/>
-    </row>
-    <row r="50" spans="1:10" s="34" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B49" s="62"/>
+      <c r="C49" s="62"/>
+      <c r="D49" s="62"/>
+      <c r="E49" s="62"/>
+      <c r="F49" s="62"/>
+      <c r="G49" s="62"/>
+      <c r="H49" s="62"/>
+      <c r="I49" s="62"/>
+      <c r="J49" s="63"/>
+    </row>
+    <row r="50" spans="1:10" s="32" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B50" s="1"/>
-      <c r="C50" s="58" t="s">
+      <c r="C50" s="54" t="s">
         <v>62</v>
       </c>
-      <c r="J50" s="35"/>
+      <c r="J50" s="33"/>
     </row>
     <row r="51" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="C51" s="53" t="s">
+      <c r="C51" s="51" t="s">
         <v>16</v>
       </c>
       <c r="D51" s="3" t="s">
@@ -2227,25 +2164,25 @@
       <c r="I51" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="J51" s="35" t="s">
+      <c r="J51" s="33" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="52" spans="1:10" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="55" t="s">
+      <c r="A52" s="53" t="s">
         <v>56</v>
       </c>
-      <c r="B52" s="51" t="s">
+      <c r="B52" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="C52" s="23"/>
-      <c r="D52" s="23"/>
-      <c r="E52" s="23"/>
-      <c r="F52" s="23"/>
-      <c r="G52" s="23"/>
-      <c r="H52" s="23"/>
-      <c r="I52" s="23"/>
-      <c r="J52" s="25">
+      <c r="C52" s="22"/>
+      <c r="D52" s="22"/>
+      <c r="E52" s="22"/>
+      <c r="F52" s="22"/>
+      <c r="G52" s="22"/>
+      <c r="H52" s="22"/>
+      <c r="I52" s="22"/>
+      <c r="J52" s="24">
         <f>SUM(C52:I52)</f>
         <v>0</v>
       </c>
@@ -2254,14 +2191,14 @@
       <c r="B53" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C53" s="23"/>
-      <c r="D53" s="23"/>
-      <c r="E53" s="23"/>
-      <c r="F53" s="23"/>
-      <c r="G53" s="23"/>
-      <c r="H53" s="23"/>
-      <c r="I53" s="23"/>
-      <c r="J53" s="25">
+      <c r="C53" s="22"/>
+      <c r="D53" s="22"/>
+      <c r="E53" s="22"/>
+      <c r="F53" s="22"/>
+      <c r="G53" s="22"/>
+      <c r="H53" s="22"/>
+      <c r="I53" s="22"/>
+      <c r="J53" s="24">
         <f t="shared" ref="J53:J58" si="7">SUM(C53:I53)</f>
         <v>0</v>
       </c>
@@ -2270,14 +2207,14 @@
       <c r="B54" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C54" s="23"/>
-      <c r="D54" s="23"/>
-      <c r="E54" s="23"/>
-      <c r="F54" s="23"/>
-      <c r="G54" s="23"/>
-      <c r="H54" s="23"/>
-      <c r="I54" s="23"/>
-      <c r="J54" s="25">
+      <c r="C54" s="22"/>
+      <c r="D54" s="22"/>
+      <c r="E54" s="22"/>
+      <c r="F54" s="22"/>
+      <c r="G54" s="22"/>
+      <c r="H54" s="22"/>
+      <c r="I54" s="22"/>
+      <c r="J54" s="24">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -2286,14 +2223,14 @@
       <c r="B55" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C55" s="23"/>
-      <c r="D55" s="23"/>
-      <c r="E55" s="23"/>
-      <c r="F55" s="23"/>
-      <c r="G55" s="23"/>
-      <c r="H55" s="23"/>
-      <c r="I55" s="23"/>
-      <c r="J55" s="25">
+      <c r="C55" s="22"/>
+      <c r="D55" s="22"/>
+      <c r="E55" s="22"/>
+      <c r="F55" s="22"/>
+      <c r="G55" s="22"/>
+      <c r="H55" s="22"/>
+      <c r="I55" s="22"/>
+      <c r="J55" s="24">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -2302,14 +2239,14 @@
       <c r="B56" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C56" s="23"/>
-      <c r="D56" s="23"/>
-      <c r="E56" s="23"/>
-      <c r="F56" s="23"/>
-      <c r="G56" s="23"/>
-      <c r="H56" s="23"/>
-      <c r="I56" s="23"/>
-      <c r="J56" s="25">
+      <c r="C56" s="22"/>
+      <c r="D56" s="22"/>
+      <c r="E56" s="22"/>
+      <c r="F56" s="22"/>
+      <c r="G56" s="22"/>
+      <c r="H56" s="22"/>
+      <c r="I56" s="22"/>
+      <c r="J56" s="24">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -2318,14 +2255,14 @@
       <c r="B57" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C57" s="23"/>
-      <c r="D57" s="23"/>
-      <c r="E57" s="23"/>
-      <c r="F57" s="23"/>
-      <c r="G57" s="23"/>
-      <c r="H57" s="23"/>
-      <c r="I57" s="23"/>
-      <c r="J57" s="25">
+      <c r="C57" s="22"/>
+      <c r="D57" s="22"/>
+      <c r="E57" s="22"/>
+      <c r="F57" s="22"/>
+      <c r="G57" s="22"/>
+      <c r="H57" s="22"/>
+      <c r="I57" s="22"/>
+      <c r="J57" s="24">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -2334,14 +2271,14 @@
       <c r="B58" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C58" s="23"/>
-      <c r="D58" s="23"/>
-      <c r="E58" s="23"/>
-      <c r="F58" s="23"/>
-      <c r="G58" s="23"/>
-      <c r="H58" s="23"/>
-      <c r="I58" s="23"/>
-      <c r="J58" s="25">
+      <c r="C58" s="22"/>
+      <c r="D58" s="22"/>
+      <c r="E58" s="22"/>
+      <c r="F58" s="22"/>
+      <c r="G58" s="22"/>
+      <c r="H58" s="22"/>
+      <c r="I58" s="22"/>
+      <c r="J58" s="24">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
@@ -2351,62 +2288,62 @@
       <c r="B59" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C59" s="25">
+      <c r="C59" s="24">
         <f>SUM(C52:C58)</f>
         <v>0</v>
       </c>
-      <c r="D59" s="25">
+      <c r="D59" s="24">
         <f t="shared" ref="D59:J59" si="8">SUM(D52:D58)</f>
         <v>0</v>
       </c>
-      <c r="E59" s="25">
+      <c r="E59" s="24">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="F59" s="25">
+      <c r="F59" s="24">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="G59" s="25">
+      <c r="G59" s="24">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="H59" s="25">
+      <c r="H59" s="24">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="I59" s="25">
+      <c r="I59" s="24">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-      <c r="J59" s="24">
+      <c r="J59" s="23">
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:10" s="34" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="62" t="s">
+    <row r="61" spans="1:10" s="32" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="58" t="s">
         <v>40</v>
       </c>
-      <c r="B61" s="63"/>
-      <c r="C61" s="63"/>
-      <c r="D61" s="63"/>
-      <c r="E61" s="63"/>
-      <c r="F61" s="63"/>
-      <c r="G61" s="63"/>
-      <c r="H61" s="63"/>
-      <c r="I61" s="63"/>
-      <c r="J61" s="64"/>
-    </row>
-    <row r="62" spans="1:10" s="34" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B61" s="59"/>
+      <c r="C61" s="59"/>
+      <c r="D61" s="59"/>
+      <c r="E61" s="59"/>
+      <c r="F61" s="59"/>
+      <c r="G61" s="59"/>
+      <c r="H61" s="59"/>
+      <c r="I61" s="59"/>
+      <c r="J61" s="60"/>
+    </row>
+    <row r="62" spans="1:10" s="32" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B62" s="1"/>
-      <c r="C62" s="58" t="s">
+      <c r="C62" s="54" t="s">
         <v>62</v>
       </c>
-      <c r="J62" s="35"/>
+      <c r="J62" s="33"/>
     </row>
     <row r="63" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="C63" s="53" t="s">
+      <c r="C63" s="51" t="s">
         <v>16</v>
       </c>
       <c r="D63" s="3" t="s">
@@ -2427,25 +2364,25 @@
       <c r="I63" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="J63" s="35" t="s">
+      <c r="J63" s="33" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="64" spans="1:10" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="55" t="s">
+      <c r="A64" s="53" t="s">
         <v>56</v>
       </c>
-      <c r="B64" s="51" t="s">
+      <c r="B64" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="C64" s="23"/>
-      <c r="D64" s="23"/>
-      <c r="E64" s="23"/>
-      <c r="F64" s="23"/>
-      <c r="G64" s="23"/>
-      <c r="H64" s="23"/>
-      <c r="I64" s="23"/>
-      <c r="J64" s="25">
+      <c r="C64" s="22"/>
+      <c r="D64" s="22"/>
+      <c r="E64" s="22"/>
+      <c r="F64" s="22"/>
+      <c r="G64" s="22"/>
+      <c r="H64" s="22"/>
+      <c r="I64" s="22"/>
+      <c r="J64" s="24">
         <f>SUM(C64:I64)</f>
         <v>0</v>
       </c>
@@ -2454,14 +2391,14 @@
       <c r="B65" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C65" s="23"/>
-      <c r="D65" s="23"/>
-      <c r="E65" s="23"/>
-      <c r="F65" s="23"/>
-      <c r="G65" s="23"/>
-      <c r="H65" s="23"/>
-      <c r="I65" s="23"/>
-      <c r="J65" s="25">
+      <c r="C65" s="22"/>
+      <c r="D65" s="22"/>
+      <c r="E65" s="22"/>
+      <c r="F65" s="22"/>
+      <c r="G65" s="22"/>
+      <c r="H65" s="22"/>
+      <c r="I65" s="22"/>
+      <c r="J65" s="24">
         <f t="shared" ref="J65:J70" si="9">SUM(C65:I65)</f>
         <v>0</v>
       </c>
@@ -2470,14 +2407,14 @@
       <c r="B66" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C66" s="23"/>
-      <c r="D66" s="23"/>
-      <c r="E66" s="23"/>
-      <c r="F66" s="23"/>
-      <c r="G66" s="23"/>
-      <c r="H66" s="23"/>
-      <c r="I66" s="23"/>
-      <c r="J66" s="25">
+      <c r="C66" s="22"/>
+      <c r="D66" s="22"/>
+      <c r="E66" s="22"/>
+      <c r="F66" s="22"/>
+      <c r="G66" s="22"/>
+      <c r="H66" s="22"/>
+      <c r="I66" s="22"/>
+      <c r="J66" s="24">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -2486,14 +2423,14 @@
       <c r="B67" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C67" s="23"/>
-      <c r="D67" s="23"/>
-      <c r="E67" s="23"/>
-      <c r="F67" s="23"/>
-      <c r="G67" s="23"/>
-      <c r="H67" s="23"/>
-      <c r="I67" s="23"/>
-      <c r="J67" s="25">
+      <c r="C67" s="22"/>
+      <c r="D67" s="22"/>
+      <c r="E67" s="22"/>
+      <c r="F67" s="22"/>
+      <c r="G67" s="22"/>
+      <c r="H67" s="22"/>
+      <c r="I67" s="22"/>
+      <c r="J67" s="24">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -2502,14 +2439,14 @@
       <c r="B68" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C68" s="23"/>
-      <c r="D68" s="23"/>
-      <c r="E68" s="23"/>
-      <c r="F68" s="23"/>
-      <c r="G68" s="23"/>
-      <c r="H68" s="23"/>
-      <c r="I68" s="23"/>
-      <c r="J68" s="25">
+      <c r="C68" s="22"/>
+      <c r="D68" s="22"/>
+      <c r="E68" s="22"/>
+      <c r="F68" s="22"/>
+      <c r="G68" s="22"/>
+      <c r="H68" s="22"/>
+      <c r="I68" s="22"/>
+      <c r="J68" s="24">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -2518,14 +2455,14 @@
       <c r="B69" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C69" s="23"/>
-      <c r="D69" s="23"/>
-      <c r="E69" s="23"/>
-      <c r="F69" s="23"/>
-      <c r="G69" s="23"/>
-      <c r="H69" s="23"/>
-      <c r="I69" s="23"/>
-      <c r="J69" s="25">
+      <c r="C69" s="22"/>
+      <c r="D69" s="22"/>
+      <c r="E69" s="22"/>
+      <c r="F69" s="22"/>
+      <c r="G69" s="22"/>
+      <c r="H69" s="22"/>
+      <c r="I69" s="22"/>
+      <c r="J69" s="24">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -2534,14 +2471,14 @@
       <c r="B70" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C70" s="23"/>
-      <c r="D70" s="23"/>
-      <c r="E70" s="23"/>
-      <c r="F70" s="23"/>
-      <c r="G70" s="23"/>
-      <c r="H70" s="23"/>
-      <c r="I70" s="23"/>
-      <c r="J70" s="25">
+      <c r="C70" s="22"/>
+      <c r="D70" s="22"/>
+      <c r="E70" s="22"/>
+      <c r="F70" s="22"/>
+      <c r="G70" s="22"/>
+      <c r="H70" s="22"/>
+      <c r="I70" s="22"/>
+      <c r="J70" s="24">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
@@ -2551,62 +2488,62 @@
       <c r="B71" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C71" s="25">
+      <c r="C71" s="24">
         <f>SUM(C64:C70)</f>
         <v>0</v>
       </c>
-      <c r="D71" s="25">
+      <c r="D71" s="24">
         <f t="shared" ref="D71:J71" si="10">SUM(D64:D70)</f>
         <v>0</v>
       </c>
-      <c r="E71" s="25">
+      <c r="E71" s="24">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="F71" s="25">
+      <c r="F71" s="24">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="G71" s="25">
+      <c r="G71" s="24">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="H71" s="25">
+      <c r="H71" s="24">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="I71" s="25">
+      <c r="I71" s="24">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="J71" s="24">
+      <c r="J71" s="23">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:10" s="34" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="59" t="s">
+    <row r="73" spans="1:10" s="32" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="55" t="s">
         <v>45</v>
       </c>
-      <c r="B73" s="60"/>
-      <c r="C73" s="60"/>
-      <c r="D73" s="60"/>
-      <c r="E73" s="60"/>
-      <c r="F73" s="60"/>
-      <c r="G73" s="60"/>
-      <c r="H73" s="60"/>
-      <c r="I73" s="60"/>
-      <c r="J73" s="61"/>
-    </row>
-    <row r="74" spans="1:10" s="34" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B73" s="56"/>
+      <c r="C73" s="56"/>
+      <c r="D73" s="56"/>
+      <c r="E73" s="56"/>
+      <c r="F73" s="56"/>
+      <c r="G73" s="56"/>
+      <c r="H73" s="56"/>
+      <c r="I73" s="56"/>
+      <c r="J73" s="57"/>
+    </row>
+    <row r="74" spans="1:10" s="32" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B74" s="1"/>
-      <c r="C74" s="58" t="s">
+      <c r="C74" s="54" t="s">
         <v>62</v>
       </c>
-      <c r="J74" s="35"/>
+      <c r="J74" s="33"/>
     </row>
     <row r="75" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="C75" s="53" t="s">
+      <c r="C75" s="51" t="s">
         <v>16</v>
       </c>
       <c r="D75" s="3" t="s">
@@ -2627,25 +2564,25 @@
       <c r="I75" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="J75" s="35" t="s">
+      <c r="J75" s="33" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="76" spans="1:10" ht="29.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="55" t="s">
+      <c r="A76" s="53" t="s">
         <v>56</v>
       </c>
-      <c r="B76" s="51" t="s">
+      <c r="B76" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="C76" s="23"/>
-      <c r="D76" s="23"/>
-      <c r="E76" s="23"/>
-      <c r="F76" s="23"/>
-      <c r="G76" s="23"/>
-      <c r="H76" s="23"/>
-      <c r="I76" s="23"/>
-      <c r="J76" s="25">
+      <c r="C76" s="22"/>
+      <c r="D76" s="22"/>
+      <c r="E76" s="22"/>
+      <c r="F76" s="22"/>
+      <c r="G76" s="22"/>
+      <c r="H76" s="22"/>
+      <c r="I76" s="22"/>
+      <c r="J76" s="24">
         <f>SUM(C76:I76)</f>
         <v>0</v>
       </c>
@@ -2654,14 +2591,14 @@
       <c r="B77" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C77" s="23"/>
-      <c r="D77" s="23"/>
-      <c r="E77" s="23"/>
-      <c r="F77" s="23"/>
-      <c r="G77" s="23"/>
-      <c r="H77" s="23"/>
-      <c r="I77" s="23"/>
-      <c r="J77" s="25">
+      <c r="C77" s="22"/>
+      <c r="D77" s="22"/>
+      <c r="E77" s="22"/>
+      <c r="F77" s="22"/>
+      <c r="G77" s="22"/>
+      <c r="H77" s="22"/>
+      <c r="I77" s="22"/>
+      <c r="J77" s="24">
         <f t="shared" ref="J77:J82" si="11">SUM(C77:I77)</f>
         <v>0</v>
       </c>
@@ -2670,14 +2607,14 @@
       <c r="B78" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C78" s="23"/>
-      <c r="D78" s="23"/>
-      <c r="E78" s="23"/>
-      <c r="F78" s="23"/>
-      <c r="G78" s="23"/>
-      <c r="H78" s="23"/>
-      <c r="I78" s="23"/>
-      <c r="J78" s="25">
+      <c r="C78" s="22"/>
+      <c r="D78" s="22"/>
+      <c r="E78" s="22"/>
+      <c r="F78" s="22"/>
+      <c r="G78" s="22"/>
+      <c r="H78" s="22"/>
+      <c r="I78" s="22"/>
+      <c r="J78" s="24">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
@@ -2686,14 +2623,14 @@
       <c r="B79" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C79" s="23"/>
-      <c r="D79" s="23"/>
-      <c r="E79" s="23"/>
-      <c r="F79" s="23"/>
-      <c r="G79" s="23"/>
-      <c r="H79" s="23"/>
-      <c r="I79" s="23"/>
-      <c r="J79" s="25">
+      <c r="C79" s="22"/>
+      <c r="D79" s="22"/>
+      <c r="E79" s="22"/>
+      <c r="F79" s="22"/>
+      <c r="G79" s="22"/>
+      <c r="H79" s="22"/>
+      <c r="I79" s="22"/>
+      <c r="J79" s="24">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
@@ -2702,14 +2639,14 @@
       <c r="B80" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C80" s="23"/>
-      <c r="D80" s="23"/>
-      <c r="E80" s="23"/>
-      <c r="F80" s="23"/>
-      <c r="G80" s="23"/>
-      <c r="H80" s="23"/>
-      <c r="I80" s="23"/>
-      <c r="J80" s="25">
+      <c r="C80" s="22"/>
+      <c r="D80" s="22"/>
+      <c r="E80" s="22"/>
+      <c r="F80" s="22"/>
+      <c r="G80" s="22"/>
+      <c r="H80" s="22"/>
+      <c r="I80" s="22"/>
+      <c r="J80" s="24">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
@@ -2718,14 +2655,14 @@
       <c r="B81" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C81" s="23"/>
-      <c r="D81" s="23"/>
-      <c r="E81" s="23"/>
-      <c r="F81" s="23"/>
-      <c r="G81" s="23"/>
-      <c r="H81" s="23"/>
-      <c r="I81" s="23"/>
-      <c r="J81" s="25">
+      <c r="C81" s="22"/>
+      <c r="D81" s="22"/>
+      <c r="E81" s="22"/>
+      <c r="F81" s="22"/>
+      <c r="G81" s="22"/>
+      <c r="H81" s="22"/>
+      <c r="I81" s="22"/>
+      <c r="J81" s="24">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
@@ -2734,14 +2671,14 @@
       <c r="B82" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C82" s="23"/>
-      <c r="D82" s="23"/>
-      <c r="E82" s="23"/>
-      <c r="F82" s="23"/>
-      <c r="G82" s="23"/>
-      <c r="H82" s="23"/>
-      <c r="I82" s="23"/>
-      <c r="J82" s="25">
+      <c r="C82" s="22"/>
+      <c r="D82" s="22"/>
+      <c r="E82" s="22"/>
+      <c r="F82" s="22"/>
+      <c r="G82" s="22"/>
+      <c r="H82" s="22"/>
+      <c r="I82" s="22"/>
+      <c r="J82" s="24">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
@@ -2751,35 +2688,35 @@
       <c r="B83" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C83" s="25">
+      <c r="C83" s="24">
         <f>SUM(C76:C82)</f>
         <v>0</v>
       </c>
-      <c r="D83" s="25">
+      <c r="D83" s="24">
         <f t="shared" ref="D83:J83" si="12">SUM(D76:D82)</f>
         <v>0</v>
       </c>
-      <c r="E83" s="25">
+      <c r="E83" s="24">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="F83" s="25">
+      <c r="F83" s="24">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="G83" s="25">
+      <c r="G83" s="24">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="H83" s="25">
+      <c r="H83" s="24">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="I83" s="25">
+      <c r="I83" s="24">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="J83" s="24">
+      <c r="J83" s="23">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
@@ -2796,421 +2733,296 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="14.5703125" customWidth="1"/>
-    <col min="3" max="10" width="15.5703125" customWidth="1"/>
+    <col min="3" max="8" width="15.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4"/>
     </row>
-    <row r="3" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="87" t="s">
+    <row r="3" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="76" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="89"/>
-      <c r="C3" s="89"/>
-      <c r="D3" s="89"/>
-      <c r="E3" s="89"/>
-      <c r="F3" s="89"/>
-      <c r="G3" s="89"/>
-      <c r="H3" s="89"/>
-      <c r="I3" s="89"/>
-      <c r="J3" s="89"/>
-    </row>
-    <row r="4" spans="1:10" ht="30.75" x14ac:dyDescent="0.3">
+      <c r="B3" s="77"/>
+      <c r="C3" s="77"/>
+      <c r="D3" s="77"/>
+      <c r="E3" s="77"/>
+      <c r="F3" s="77"/>
+      <c r="G3" s="77"/>
+      <c r="H3" s="77"/>
+    </row>
+    <row r="4" spans="1:8" ht="30.75" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
-      <c r="F4" s="43" t="s">
+      <c r="F4" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="G4" s="43" t="s">
+      <c r="G4" s="41" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
-      <c r="C5" s="34"/>
-      <c r="D5" s="34"/>
-      <c r="E5" s="28" t="s">
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="F5" s="41">
+      <c r="F5" s="39">
         <f>SUM(F6:F9)</f>
         <v>0</v>
       </c>
-      <c r="G5" s="44" t="e">
+      <c r="G5" s="42" t="e">
         <f>SUM(G6:G9)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H5" s="34"/>
-      <c r="I5" s="34"/>
-      <c r="J5" s="35"/>
-    </row>
-    <row r="6" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="H5" s="32"/>
+    </row>
+    <row r="6" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
-      <c r="C6" s="34"/>
-      <c r="D6" s="34"/>
-      <c r="E6" s="28" t="s">
+      <c r="C6" s="32"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="F6" s="45"/>
-      <c r="G6" s="46" t="e">
+      <c r="F6" s="43"/>
+      <c r="G6" s="44" t="e">
         <f>F6/$F$5</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H6" s="34"/>
-      <c r="I6" s="34"/>
-      <c r="J6" s="35"/>
-    </row>
-    <row r="7" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="H6" s="32"/>
+    </row>
+    <row r="7" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
-      <c r="C7" s="34"/>
-      <c r="D7" s="34"/>
-      <c r="E7" s="28" t="s">
+      <c r="C7" s="32"/>
+      <c r="D7" s="32"/>
+      <c r="E7" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="42"/>
-      <c r="G7" s="29" t="e">
-        <f t="shared" ref="G7:G9" si="0">F7/$F$5</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H7" s="34"/>
-      <c r="I7" s="34"/>
-      <c r="J7" s="35"/>
-    </row>
-    <row r="8" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="F7" s="40"/>
+      <c r="G7" s="28" t="e">
+        <f>F7/$F$5</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H7" s="32"/>
+    </row>
+    <row r="8" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
-      <c r="C8" s="34"/>
-      <c r="D8" s="34"/>
-      <c r="E8" s="28" t="s">
+      <c r="C8" s="32"/>
+      <c r="D8" s="32"/>
+      <c r="E8" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="F8" s="49"/>
-      <c r="G8" s="50" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H8" s="34"/>
-      <c r="I8" s="34"/>
-      <c r="J8" s="35"/>
-    </row>
-    <row r="9" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="F8" s="47"/>
+      <c r="G8" s="48" t="e">
+        <f>F8/$F$5</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H8" s="32"/>
+    </row>
+    <row r="9" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
-      <c r="C9" s="34"/>
-      <c r="D9" s="34"/>
-      <c r="E9" s="28" t="s">
+      <c r="C9" s="32"/>
+      <c r="D9" s="32"/>
+      <c r="E9" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="F9" s="47"/>
-      <c r="G9" s="48" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H9" s="34"/>
-      <c r="I9" s="34"/>
-      <c r="J9" s="35"/>
-    </row>
-    <row r="10" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F9" s="45"/>
+      <c r="G9" s="46" t="e">
+        <f>F9/$F$5</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H9" s="32"/>
+    </row>
+    <row r="10" spans="1:8" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
     </row>
-    <row r="11" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4"/>
-      <c r="F11" s="27" t="s">
-        <v>65</v>
-      </c>
-      <c r="G11" s="31" t="e">
+      <c r="F11" s="26" t="s">
+        <v>64</v>
+      </c>
+      <c r="G11" s="30" t="e">
         <f>#REF!/G22</f>
         <v>#REF!</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4"/>
     </row>
-    <row r="13" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="78" t="s">
-        <v>66</v>
-      </c>
-      <c r="B13" s="78"/>
-      <c r="C13" s="78"/>
-      <c r="D13" s="78"/>
-      <c r="E13" s="78"/>
-      <c r="F13" s="78"/>
-      <c r="G13" s="78"/>
-      <c r="H13" s="78"/>
-      <c r="I13" s="78"/>
-      <c r="J13" s="78"/>
-    </row>
-    <row r="14" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="79" t="s">
+        <v>65</v>
+      </c>
+      <c r="B13" s="79"/>
+      <c r="C13" s="79"/>
+      <c r="D13" s="79"/>
+      <c r="E13" s="79"/>
+      <c r="F13" s="79"/>
+      <c r="G13" s="79"/>
+      <c r="H13" s="79"/>
+    </row>
+    <row r="14" spans="1:8" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4"/>
     </row>
-    <row r="15" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C15" s="17" t="s">
+    <row r="15" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C15" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="D15" s="17" t="s">
+      <c r="D15" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="E15" s="17" t="s">
+      <c r="E15" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="F15" s="17" t="s">
+      <c r="F15" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="G15" s="17" t="s">
+      <c r="G15" s="16" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="79"/>
-      <c r="B16" s="51" t="s">
+    <row r="16" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="70"/>
+      <c r="B16" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="26" t="e">
+      <c r="C16" s="25" t="e">
         <f>G16/(E16*100)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D16" s="26" t="e">
+      <c r="D16" s="25" t="e">
         <f>#REF!/(F16*100)</f>
         <v>#REF!</v>
       </c>
-      <c r="E16" s="26"/>
-      <c r="F16" s="26"/>
-      <c r="G16" s="26"/>
-    </row>
-    <row r="17" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E16" s="25"/>
+      <c r="F16" s="25"/>
+      <c r="G16" s="25"/>
+    </row>
+    <row r="17" spans="1:8" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C17" s="26" t="e">
-        <f t="shared" ref="C17:C21" si="1">G17/(E17*100)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D17" s="26" t="e">
+      <c r="C17" s="25" t="e">
+        <f t="shared" ref="C17:C21" si="0">G17/(E17*100)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D17" s="25" t="e">
         <f>#REF!/(F17*100)</f>
         <v>#REF!</v>
       </c>
-      <c r="E17" s="26"/>
-      <c r="F17" s="26"/>
-      <c r="G17" s="26"/>
-    </row>
-    <row r="18" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E17" s="25"/>
+      <c r="F17" s="25"/>
+      <c r="G17" s="25"/>
+    </row>
+    <row r="18" spans="1:8" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C18" s="26" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D18" s="26" t="e">
+      <c r="C18" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D18" s="25" t="e">
         <f>#REF!/(F18*100)</f>
         <v>#REF!</v>
       </c>
-      <c r="E18" s="26"/>
-      <c r="F18" s="26"/>
-      <c r="G18" s="26"/>
-    </row>
-    <row r="19" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E18" s="25"/>
+      <c r="F18" s="25"/>
+      <c r="G18" s="25"/>
+    </row>
+    <row r="19" spans="1:8" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C19" s="26" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D19" s="26" t="e">
+      <c r="C19" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D19" s="25" t="e">
         <f>#REF!/(F19*100)</f>
         <v>#REF!</v>
       </c>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
-    </row>
-    <row r="20" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E19" s="25"/>
+      <c r="F19" s="25"/>
+      <c r="G19" s="25"/>
+    </row>
+    <row r="20" spans="1:8" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C20" s="26" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D20" s="26" t="e">
+      <c r="C20" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D20" s="25" t="e">
         <f>#REF!/(F20*100)</f>
         <v>#REF!</v>
       </c>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
-      <c r="G20" s="26"/>
-    </row>
-    <row r="21" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E20" s="25"/>
+      <c r="F20" s="25"/>
+      <c r="G20" s="25"/>
+    </row>
+    <row r="21" spans="1:8" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C21" s="26" t="e">
-        <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="D21" s="26" t="e">
+      <c r="C21" s="25" t="e">
+        <f t="shared" si="0"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D21" s="25" t="e">
         <f>#REF!/(F21*100)</f>
         <v>#REF!</v>
       </c>
-      <c r="E21" s="26"/>
-      <c r="F21" s="26"/>
-      <c r="G21" s="26"/>
-    </row>
-    <row r="22" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E21" s="25"/>
+      <c r="F21" s="25"/>
+      <c r="G21" s="25"/>
+    </row>
+    <row r="22" spans="1:8" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="9"/>
-      <c r="C22" s="25"/>
+      <c r="C22" s="24"/>
       <c r="D22" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E22" s="25">
+      <c r="E22" s="24">
         <f>SUM(E16:E21)</f>
         <v>0</v>
       </c>
-      <c r="F22" s="25">
+      <c r="F22" s="24">
         <f>SUM(F16:F21)</f>
         <v>0</v>
       </c>
-      <c r="G22" s="25">
+      <c r="G22" s="24">
         <f>SUM(G16:G21)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:9" s="34" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="73" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" s="34" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="1"/>
-      <c r="C25" s="56" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="B26" s="34"/>
-      <c r="C26" s="32" t="s">
-        <v>16</v>
-      </c>
-      <c r="D26" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="E26" s="16" t="s">
-        <v>5</v>
-      </c>
-      <c r="F26" s="16" t="s">
-        <v>6</v>
-      </c>
-      <c r="G26" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="H26" s="16" t="s">
-        <v>39</v>
-      </c>
-      <c r="I26" s="34"/>
-    </row>
-    <row r="27" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="57" t="s">
-        <v>56</v>
-      </c>
-      <c r="B27" s="75" t="s">
-        <v>16</v>
-      </c>
-      <c r="C27" s="76"/>
-      <c r="D27" s="76"/>
-      <c r="E27" s="76"/>
-      <c r="F27" s="76"/>
-      <c r="G27" s="76"/>
-      <c r="H27" s="76"/>
-      <c r="I27" s="81"/>
-    </row>
-    <row r="28" spans="1:9" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="77" t="s">
-        <v>4</v>
-      </c>
-      <c r="C28" s="76"/>
-      <c r="D28" s="76"/>
-      <c r="E28" s="76"/>
-      <c r="F28" s="76"/>
-      <c r="G28" s="76"/>
-      <c r="H28" s="76"/>
-      <c r="I28" s="81"/>
-    </row>
-    <row r="29" spans="1:9" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="77" t="s">
-        <v>5</v>
-      </c>
-      <c r="C29" s="76"/>
-      <c r="D29" s="76"/>
-      <c r="E29" s="76"/>
-      <c r="F29" s="76"/>
-      <c r="G29" s="76"/>
-      <c r="H29" s="76"/>
-      <c r="I29" s="81"/>
-    </row>
-    <row r="30" spans="1:9" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="77" t="s">
-        <v>6</v>
-      </c>
-      <c r="C30" s="76"/>
-      <c r="D30" s="76"/>
-      <c r="E30" s="76"/>
-      <c r="F30" s="76"/>
-      <c r="G30" s="76"/>
-      <c r="H30" s="76"/>
-      <c r="I30" s="81"/>
-    </row>
-    <row r="31" spans="1:9" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="77" t="s">
-        <v>7</v>
-      </c>
-      <c r="C31" s="76"/>
-      <c r="D31" s="76"/>
-      <c r="E31" s="76"/>
-      <c r="F31" s="76"/>
-      <c r="G31" s="76"/>
-      <c r="H31" s="76"/>
-      <c r="I31" s="81"/>
-    </row>
-    <row r="32" spans="1:9" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="77" t="s">
-        <v>39</v>
-      </c>
-      <c r="C32" s="76"/>
-      <c r="D32" s="76"/>
-      <c r="E32" s="76"/>
-      <c r="F32" s="76"/>
-      <c r="G32" s="76"/>
-      <c r="H32" s="76"/>
-      <c r="I32" s="81"/>
-    </row>
-    <row r="33" spans="1:10" s="37" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="8"/>
-      <c r="B33" s="35"/>
-      <c r="C33" s="80"/>
-      <c r="D33" s="80"/>
-      <c r="E33" s="80"/>
-      <c r="F33" s="80"/>
-      <c r="G33" s="80"/>
-      <c r="H33" s="80"/>
-      <c r="I33" s="35"/>
-      <c r="J33" s="35"/>
-    </row>
-    <row r="34" spans="1:10" s="37" customFormat="1" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="36" t="s">
+    <row r="24" spans="1:8" s="35" customFormat="1" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="78" t="s">
         <v>63</v>
       </c>
+      <c r="B24" s="78"/>
+      <c r="C24" s="78"/>
+      <c r="D24" s="78"/>
+      <c r="E24" s="78"/>
+      <c r="F24" s="78"/>
+      <c r="G24" s="78"/>
+      <c r="H24" s="78"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A3:J3"/>
+  <mergeCells count="3">
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A13:H13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3225,7 +3037,7 @@
     <col min="1" max="1" width="8.7109375" customWidth="1"/>
     <col min="2" max="2" width="14.5703125" customWidth="1"/>
     <col min="3" max="9" width="15.5703125" customWidth="1"/>
-    <col min="10" max="10" width="15.5703125" style="35" customWidth="1"/>
+    <col min="10" max="10" width="15.5703125" style="33" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" s="11" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.35">
@@ -3238,292 +3050,292 @@
       <c r="A2" s="4"/>
     </row>
     <row r="3" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="87" t="s">
+      <c r="A3" s="76" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="89"/>
-      <c r="C3" s="89"/>
-      <c r="D3" s="89"/>
-      <c r="E3" s="89"/>
-      <c r="F3" s="89"/>
-      <c r="G3" s="89"/>
-      <c r="H3" s="89"/>
-      <c r="I3" s="89"/>
-      <c r="J3" s="91"/>
+      <c r="B3" s="77"/>
+      <c r="C3" s="77"/>
+      <c r="D3" s="77"/>
+      <c r="E3" s="77"/>
+      <c r="F3" s="77"/>
+      <c r="G3" s="77"/>
+      <c r="H3" s="77"/>
+      <c r="I3" s="77"/>
+      <c r="J3" s="82"/>
     </row>
     <row r="4" spans="1:10" ht="30.75" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
-      <c r="F4" s="43" t="s">
+      <c r="F4" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="G4" s="43" t="s">
+      <c r="G4" s="41" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
-      <c r="C5" s="34"/>
-      <c r="D5" s="34"/>
-      <c r="E5" s="28" t="s">
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="F5" s="41">
+      <c r="F5" s="39">
         <f>SUM(F6:F9)</f>
         <v>0</v>
       </c>
-      <c r="G5" s="44" t="e">
+      <c r="G5" s="42" t="e">
         <f>SUM(G6:G9)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H5" s="34"/>
-      <c r="I5" s="34"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
     </row>
     <row r="6" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
-      <c r="C6" s="34"/>
-      <c r="D6" s="34"/>
-      <c r="E6" s="28" t="s">
+      <c r="C6" s="32"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="27" t="s">
         <v>31</v>
       </c>
-      <c r="F6" s="45"/>
-      <c r="G6" s="46" t="e">
+      <c r="F6" s="43"/>
+      <c r="G6" s="44" t="e">
         <f>F6/$F$5</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H6" s="34"/>
-      <c r="I6" s="34"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="32"/>
     </row>
     <row r="7" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
-      <c r="C7" s="34"/>
-      <c r="D7" s="34"/>
-      <c r="E7" s="28" t="s">
+      <c r="C7" s="32"/>
+      <c r="D7" s="32"/>
+      <c r="E7" s="27" t="s">
         <v>32</v>
       </c>
-      <c r="F7" s="42"/>
-      <c r="G7" s="29" t="e">
+      <c r="F7" s="40"/>
+      <c r="G7" s="28" t="e">
         <f t="shared" ref="G7:G9" si="0">F7/$F$5</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H7" s="34"/>
-      <c r="I7" s="34"/>
+      <c r="H7" s="32"/>
+      <c r="I7" s="32"/>
     </row>
     <row r="8" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
-      <c r="C8" s="34"/>
-      <c r="D8" s="34"/>
-      <c r="E8" s="28" t="s">
+      <c r="C8" s="32"/>
+      <c r="D8" s="32"/>
+      <c r="E8" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="F8" s="49"/>
-      <c r="G8" s="50" t="e">
+      <c r="F8" s="47"/>
+      <c r="G8" s="48" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="H8" s="34"/>
-      <c r="I8" s="34"/>
+      <c r="H8" s="32"/>
+      <c r="I8" s="32"/>
     </row>
     <row r="9" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
-      <c r="C9" s="34"/>
-      <c r="D9" s="34"/>
-      <c r="E9" s="28" t="s">
+      <c r="C9" s="32"/>
+      <c r="D9" s="32"/>
+      <c r="E9" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="F9" s="47"/>
-      <c r="G9" s="48" t="e">
+      <c r="F9" s="45"/>
+      <c r="G9" s="46" t="e">
         <f t="shared" si="0"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="H9" s="34"/>
-      <c r="I9" s="34"/>
+      <c r="H9" s="32"/>
+      <c r="I9" s="32"/>
     </row>
     <row r="10" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
       <c r="J10"/>
     </row>
     <row r="11" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="92" t="s">
+      <c r="A11" s="83" t="s">
         <v>35</v>
       </c>
-      <c r="B11" s="93"/>
-      <c r="C11" s="93"/>
-      <c r="D11" s="93"/>
-      <c r="E11" s="93"/>
-      <c r="F11" s="93"/>
-      <c r="G11" s="93"/>
-      <c r="H11" s="93"/>
-      <c r="I11" s="93"/>
-      <c r="J11" s="94"/>
+      <c r="B11" s="84"/>
+      <c r="C11" s="84"/>
+      <c r="D11" s="84"/>
+      <c r="E11" s="84"/>
+      <c r="F11" s="84"/>
+      <c r="G11" s="84"/>
+      <c r="H11" s="84"/>
+      <c r="I11" s="84"/>
+      <c r="J11" s="85"/>
     </row>
     <row r="12" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4"/>
       <c r="J12"/>
     </row>
     <row r="13" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C13" s="17" t="s">
+      <c r="C13" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="D13" s="17" t="s">
+      <c r="D13" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="E13" s="18" t="s">
+      <c r="E13" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="F13" s="18" t="s">
+      <c r="F13" s="17" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="79"/>
-      <c r="B14" s="51" t="s">
+      <c r="A14" s="70"/>
+      <c r="B14" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="23">
+      <c r="C14" s="22">
         <f t="shared" ref="C14:C20" si="1">J26</f>
         <v>0</v>
       </c>
-      <c r="D14" s="23">
+      <c r="D14" s="22">
         <f>C33</f>
         <v>0</v>
       </c>
-      <c r="E14" s="23">
+      <c r="E14" s="22">
         <f t="shared" ref="E14:E20" si="2">D14-C14</f>
         <v>0</v>
       </c>
-      <c r="F14" s="30" t="e">
+      <c r="F14" s="29" t="e">
         <f t="shared" ref="F14:F20" si="3">(D14-C14)/C14</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="79"/>
+      <c r="A15" s="70"/>
       <c r="B15" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C15" s="23">
+      <c r="C15" s="22">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D15" s="23">
+      <c r="D15" s="22">
         <f>D33</f>
         <v>0</v>
       </c>
-      <c r="E15" s="23">
+      <c r="E15" s="22">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="F15" s="30" t="e">
+      <c r="F15" s="29" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="79"/>
+      <c r="A16" s="70"/>
       <c r="B16" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C16" s="23">
+      <c r="C16" s="22">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D16" s="23">
+      <c r="D16" s="22">
         <f>E33</f>
         <v>0</v>
       </c>
-      <c r="E16" s="23">
+      <c r="E16" s="22">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="F16" s="30" t="e">
+      <c r="F16" s="29" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="79"/>
+      <c r="A17" s="70"/>
       <c r="B17" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C17" s="23">
+      <c r="C17" s="22">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D17" s="23">
+      <c r="D17" s="22">
         <f>F33</f>
         <v>0</v>
       </c>
-      <c r="E17" s="23">
+      <c r="E17" s="22">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="F17" s="30" t="e">
+      <c r="F17" s="29" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="79"/>
+      <c r="A18" s="70"/>
       <c r="B18" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C18" s="23">
+      <c r="C18" s="22">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D18" s="23">
+      <c r="D18" s="22">
         <f>G33</f>
         <v>0</v>
       </c>
-      <c r="E18" s="23">
+      <c r="E18" s="22">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="F18" s="30" t="e">
+      <c r="F18" s="29" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="79"/>
+      <c r="A19" s="70"/>
       <c r="B19" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C19" s="23">
+      <c r="C19" s="22">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D19" s="23">
+      <c r="D19" s="22">
         <f>H33</f>
         <v>0</v>
       </c>
-      <c r="E19" s="23">
+      <c r="E19" s="22">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="F19" s="30" t="e">
+      <c r="F19" s="29" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="79"/>
+      <c r="A20" s="70"/>
       <c r="B20" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C20" s="23">
+      <c r="C20" s="22">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="D20" s="23">
+      <c r="D20" s="22">
         <f>I33</f>
         <v>0</v>
       </c>
-      <c r="E20" s="23">
+      <c r="E20" s="22">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="F20" s="30" t="e">
+      <c r="F20" s="29" t="e">
         <f t="shared" si="3"/>
         <v>#DIV/0!</v>
       </c>
@@ -3533,77 +3345,77 @@
       <c r="B21" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C21" s="25">
+      <c r="C21" s="24">
         <f>SUM(C14:C20)</f>
         <v>0</v>
       </c>
-      <c r="D21" s="25">
+      <c r="D21" s="24">
         <f>SUM(D14:D20)</f>
         <v>0</v>
       </c>
-      <c r="E21" s="25"/>
-      <c r="F21" s="22"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="21"/>
     </row>
     <row r="22" spans="1:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4"/>
       <c r="B22" s="6"/>
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
-    </row>
-    <row r="23" spans="1:10" s="34" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="74" t="s">
+      <c r="C22" s="18"/>
+      <c r="D22" s="18"/>
+    </row>
+    <row r="23" spans="1:10" s="32" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="69" t="s">
         <v>15</v>
       </c>
-      <c r="J23" s="35"/>
-    </row>
-    <row r="24" spans="1:10" s="34" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J23" s="33"/>
+    </row>
+    <row r="24" spans="1:10" s="32" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="1"/>
-      <c r="C24" s="58" t="s">
+      <c r="C24" s="54" t="s">
         <v>62</v>
       </c>
-      <c r="J24" s="35"/>
+      <c r="J24" s="33"/>
     </row>
     <row r="25" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="C25" s="52" t="s">
+      <c r="C25" s="50" t="s">
         <v>16</v>
       </c>
-      <c r="D25" s="20" t="s">
+      <c r="D25" s="19" t="s">
         <v>4</v>
       </c>
-      <c r="E25" s="20" t="s">
+      <c r="E25" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="F25" s="20" t="s">
+      <c r="F25" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="G25" s="20" t="s">
+      <c r="G25" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="H25" s="20" t="s">
+      <c r="H25" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="I25" s="21" t="s">
+      <c r="I25" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="J25" s="35" t="s">
+      <c r="J25" s="33" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="55" t="s">
+      <c r="A26" s="53" t="s">
         <v>56</v>
       </c>
-      <c r="B26" s="51" t="s">
+      <c r="B26" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="C26" s="23"/>
-      <c r="D26" s="23"/>
-      <c r="E26" s="23"/>
-      <c r="F26" s="23"/>
-      <c r="G26" s="23"/>
-      <c r="H26" s="23"/>
-      <c r="I26" s="23"/>
-      <c r="J26" s="25">
+      <c r="C26" s="22"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="22"/>
+      <c r="F26" s="22"/>
+      <c r="G26" s="22"/>
+      <c r="H26" s="22"/>
+      <c r="I26" s="22"/>
+      <c r="J26" s="24">
         <f t="shared" ref="J26:J33" si="4">SUM(C26:I26)</f>
         <v>0</v>
       </c>
@@ -3612,14 +3424,14 @@
       <c r="B27" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C27" s="23"/>
-      <c r="D27" s="23"/>
-      <c r="E27" s="23"/>
-      <c r="F27" s="23"/>
-      <c r="G27" s="23"/>
-      <c r="H27" s="23"/>
-      <c r="I27" s="23"/>
-      <c r="J27" s="25">
+      <c r="C27" s="22"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="22"/>
+      <c r="F27" s="22"/>
+      <c r="G27" s="22"/>
+      <c r="H27" s="22"/>
+      <c r="I27" s="22"/>
+      <c r="J27" s="24">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -3628,14 +3440,14 @@
       <c r="B28" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C28" s="23"/>
-      <c r="D28" s="23"/>
-      <c r="E28" s="23"/>
-      <c r="F28" s="23"/>
-      <c r="G28" s="23"/>
-      <c r="H28" s="23"/>
-      <c r="I28" s="23"/>
-      <c r="J28" s="25">
+      <c r="C28" s="22"/>
+      <c r="D28" s="22"/>
+      <c r="E28" s="22"/>
+      <c r="F28" s="22"/>
+      <c r="G28" s="22"/>
+      <c r="H28" s="22"/>
+      <c r="I28" s="22"/>
+      <c r="J28" s="24">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -3644,14 +3456,14 @@
       <c r="B29" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C29" s="23"/>
-      <c r="D29" s="23"/>
-      <c r="E29" s="23"/>
-      <c r="F29" s="23"/>
-      <c r="G29" s="23"/>
-      <c r="H29" s="23"/>
-      <c r="I29" s="23"/>
-      <c r="J29" s="25">
+      <c r="C29" s="22"/>
+      <c r="D29" s="22"/>
+      <c r="E29" s="22"/>
+      <c r="F29" s="22"/>
+      <c r="G29" s="22"/>
+      <c r="H29" s="22"/>
+      <c r="I29" s="22"/>
+      <c r="J29" s="24">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -3660,14 +3472,14 @@
       <c r="B30" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C30" s="23"/>
-      <c r="D30" s="23"/>
-      <c r="E30" s="23"/>
-      <c r="F30" s="23"/>
-      <c r="G30" s="23"/>
-      <c r="H30" s="23"/>
-      <c r="I30" s="23"/>
-      <c r="J30" s="25">
+      <c r="C30" s="22"/>
+      <c r="D30" s="22"/>
+      <c r="E30" s="22"/>
+      <c r="F30" s="22"/>
+      <c r="G30" s="22"/>
+      <c r="H30" s="22"/>
+      <c r="I30" s="22"/>
+      <c r="J30" s="24">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -3676,14 +3488,14 @@
       <c r="B31" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C31" s="23"/>
-      <c r="D31" s="23"/>
-      <c r="E31" s="23"/>
-      <c r="F31" s="23"/>
-      <c r="G31" s="23"/>
-      <c r="H31" s="23"/>
-      <c r="I31" s="23"/>
-      <c r="J31" s="25">
+      <c r="C31" s="22"/>
+      <c r="D31" s="22"/>
+      <c r="E31" s="22"/>
+      <c r="F31" s="22"/>
+      <c r="G31" s="22"/>
+      <c r="H31" s="22"/>
+      <c r="I31" s="22"/>
+      <c r="J31" s="24">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -3692,52 +3504,52 @@
       <c r="B32" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C32" s="23"/>
-      <c r="D32" s="23"/>
-      <c r="E32" s="23"/>
-      <c r="F32" s="23"/>
-      <c r="G32" s="23"/>
-      <c r="H32" s="23"/>
-      <c r="I32" s="23"/>
-      <c r="J32" s="25">
+      <c r="C32" s="22"/>
+      <c r="D32" s="22"/>
+      <c r="E32" s="22"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="22"/>
+      <c r="H32" s="22"/>
+      <c r="I32" s="22"/>
+      <c r="J32" s="24">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:10" s="37" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" s="35" customFormat="1" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="8"/>
       <c r="B33" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C33" s="25">
+      <c r="C33" s="24">
         <f t="shared" ref="C33:I33" si="5">SUM(C26:C32)</f>
         <v>0</v>
       </c>
-      <c r="D33" s="25">
+      <c r="D33" s="24">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="E33" s="25">
+      <c r="E33" s="24">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="F33" s="25">
+      <c r="F33" s="24">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="G33" s="25">
+      <c r="G33" s="24">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="H33" s="25">
+      <c r="H33" s="24">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="I33" s="25">
+      <c r="I33" s="24">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="J33" s="24">
+      <c r="J33" s="23">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
@@ -3783,136 +3595,136 @@
       <c r="A2" s="4"/>
     </row>
     <row r="3" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A3" s="87" t="s">
+      <c r="A3" s="76" t="s">
         <v>48</v>
       </c>
-      <c r="B3" s="89"/>
-      <c r="C3" s="89"/>
-      <c r="D3" s="89"/>
-      <c r="E3" s="89"/>
-      <c r="F3" s="89"/>
-      <c r="G3" s="89"/>
-      <c r="H3" s="89"/>
-      <c r="I3" s="89"/>
-      <c r="J3" s="91"/>
+      <c r="B3" s="77"/>
+      <c r="C3" s="77"/>
+      <c r="D3" s="77"/>
+      <c r="E3" s="77"/>
+      <c r="F3" s="77"/>
+      <c r="G3" s="77"/>
+      <c r="H3" s="77"/>
+      <c r="I3" s="77"/>
+      <c r="J3" s="82"/>
     </row>
     <row r="4" spans="1:10" ht="41.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
-      <c r="D4" s="43" t="s">
+      <c r="D4" s="41" t="s">
         <v>49</v>
       </c>
-      <c r="E4" s="43" t="s">
+      <c r="E4" s="41" t="s">
         <v>38</v>
       </c>
-      <c r="F4" s="43" t="s">
+      <c r="F4" s="41" t="s">
         <v>50</v>
       </c>
-      <c r="G4" s="43" t="s">
+      <c r="G4" s="41" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
-      <c r="C5" s="28" t="s">
+      <c r="C5" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="41">
+      <c r="D5" s="39">
         <f>'SDG 15.3.1'!F5</f>
         <v>0</v>
       </c>
-      <c r="E5" s="44" t="e">
+      <c r="E5" s="42" t="e">
         <f>'SDG 15.3.1'!G5</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F5" s="82">
+      <c r="F5" s="71">
         <f>SUM(F6:F9)</f>
         <v>0</v>
       </c>
-      <c r="G5" s="44" t="e">
+      <c r="G5" s="42" t="e">
         <f>SUM(G6:G9)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="I5" s="34"/>
+      <c r="I5" s="32"/>
     </row>
     <row r="6" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
-      <c r="C6" s="28" t="s">
+      <c r="C6" s="27" t="s">
         <v>52</v>
       </c>
-      <c r="D6" s="45">
+      <c r="D6" s="43">
         <f>'SDG 15.3.1'!F6</f>
         <v>0</v>
       </c>
-      <c r="E6" s="46" t="e">
+      <c r="E6" s="44" t="e">
         <f>'SDG 15.3.1'!G6</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F6" s="83"/>
-      <c r="G6" s="46" t="e">
+      <c r="F6" s="72"/>
+      <c r="G6" s="44" t="e">
         <f>F6/F$5</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="I6" s="34"/>
+      <c r="I6" s="32"/>
     </row>
     <row r="7" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
-      <c r="C7" s="28" t="s">
+      <c r="C7" s="27" t="s">
         <v>53</v>
       </c>
-      <c r="D7" s="42">
+      <c r="D7" s="40">
         <f>'SDG 15.3.1'!F7</f>
         <v>0</v>
       </c>
-      <c r="E7" s="29" t="e">
+      <c r="E7" s="28" t="e">
         <f>'SDG 15.3.1'!G7</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F7" s="84"/>
-      <c r="G7" s="29" t="e">
+      <c r="F7" s="73"/>
+      <c r="G7" s="28" t="e">
         <f>F7/F$5</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="I7" s="34"/>
+      <c r="I7" s="32"/>
     </row>
     <row r="8" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
-      <c r="C8" s="28" t="s">
+      <c r="C8" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="D8" s="49">
+      <c r="D8" s="47">
         <f>'SDG 15.3.1'!F8</f>
         <v>0</v>
       </c>
-      <c r="E8" s="50" t="e">
+      <c r="E8" s="48" t="e">
         <f>'SDG 15.3.1'!G8</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F8" s="85"/>
-      <c r="G8" s="50" t="e">
+      <c r="F8" s="74"/>
+      <c r="G8" s="48" t="e">
         <f>F8/F$5</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="I8" s="34"/>
+      <c r="I8" s="32"/>
     </row>
     <row r="9" spans="1:10" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
-      <c r="C9" s="28" t="s">
+      <c r="C9" s="27" t="s">
         <v>54</v>
       </c>
-      <c r="D9" s="47">
+      <c r="D9" s="45">
         <f>'SDG 15.3.1'!F9</f>
         <v>0</v>
       </c>
-      <c r="E9" s="48" t="e">
+      <c r="E9" s="46" t="e">
         <f>'SDG 15.3.1'!G9</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="F9" s="86"/>
-      <c r="G9" s="48" t="e">
+      <c r="F9" s="75"/>
+      <c r="G9" s="46" t="e">
         <f>F9/F$5</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="I9" s="34"/>
+      <c r="I9" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Fix soc table template and use formulas in template for change/pct change
</commit_message>
<xml_diff>
--- a/te_algorithms/data/summary_table_ld_sdg.xlsx
+++ b/te_algorithms/data/summary_table_ld_sdg.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-26.04\home\azvoleff\Code\LandDegradation\trends.earth-algorithms\te_algorithms\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3251D70C-8223-45A5-BB8B-12CE3F5B6775}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF4BC7F9-4A64-411D-89C4-95054B41CAA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SDG 15.3.1" sheetId="5" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="70">
   <si>
     <t>Land area with improved productivity:</t>
   </si>
@@ -238,6 +238,12 @@
   </si>
   <si>
     <t>* For the SDG indicator, areas are considered to be improved if they have "Improving" productivity, to be stable if they have "stable" or "stressed" productivity, and to be "degraded" if they are classified as in "moderate decline" or "declining".</t>
+  </si>
+  <si>
+    <t>Change in soil organic carbon (tonnes)</t>
+  </si>
+  <si>
+    <t>Change in soil organic carbon (percent)</t>
   </si>
 </sst>
 </file>
@@ -248,7 +254,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -398,6 +404,11 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="13">
     <fill>
@@ -667,7 +678,7 @@
     <xf numFmtId="43" fontId="8" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -887,20 +898,20 @@
     <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -908,6 +919,12 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="15" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1355,18 +1372,18 @@
       <c r="A10" s="4"/>
     </row>
     <row r="11" spans="1:10" s="34" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="80" t="s">
+      <c r="A11" s="77" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="80"/>
-      <c r="C11" s="80"/>
-      <c r="D11" s="80"/>
-      <c r="E11" s="80"/>
-      <c r="F11" s="80"/>
-      <c r="G11" s="80"/>
-      <c r="H11" s="80"/>
-      <c r="I11" s="80"/>
-      <c r="J11" s="80"/>
+      <c r="B11" s="77"/>
+      <c r="C11" s="77"/>
+      <c r="D11" s="77"/>
+      <c r="E11" s="77"/>
+      <c r="F11" s="77"/>
+      <c r="G11" s="77"/>
+      <c r="H11" s="77"/>
+      <c r="I11" s="77"/>
+      <c r="J11" s="77"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="31" t="s">
@@ -1422,15 +1439,15 @@
       <c r="A3" s="76" t="s">
         <v>46</v>
       </c>
-      <c r="B3" s="77"/>
-      <c r="C3" s="77"/>
-      <c r="D3" s="77"/>
-      <c r="E3" s="77"/>
-      <c r="F3" s="77"/>
-      <c r="G3" s="77"/>
-      <c r="H3" s="77"/>
-      <c r="I3" s="77"/>
-      <c r="J3" s="77"/>
+      <c r="B3" s="78"/>
+      <c r="C3" s="78"/>
+      <c r="D3" s="78"/>
+      <c r="E3" s="78"/>
+      <c r="F3" s="78"/>
+      <c r="G3" s="78"/>
+      <c r="H3" s="78"/>
+      <c r="I3" s="78"/>
+      <c r="J3" s="78"/>
     </row>
     <row r="4" spans="1:10" ht="30.75" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
@@ -1503,18 +1520,18 @@
       <c r="A10" s="4"/>
     </row>
     <row r="11" spans="1:10" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="80" t="s">
+      <c r="A11" s="77" t="s">
         <v>67</v>
       </c>
-      <c r="B11" s="77"/>
-      <c r="C11" s="81"/>
-      <c r="D11" s="81"/>
-      <c r="E11" s="81"/>
-      <c r="F11" s="81"/>
-      <c r="G11" s="81"/>
-      <c r="H11" s="81"/>
-      <c r="I11" s="81"/>
-      <c r="J11" s="82"/>
+      <c r="B11" s="78"/>
+      <c r="C11" s="79"/>
+      <c r="D11" s="79"/>
+      <c r="E11" s="79"/>
+      <c r="F11" s="79"/>
+      <c r="G11" s="79"/>
+      <c r="H11" s="79"/>
+      <c r="I11" s="79"/>
+      <c r="J11" s="80"/>
     </row>
     <row r="12" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4"/>
@@ -2733,34 +2750,35 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="14.5703125" customWidth="1"/>
-    <col min="3" max="8" width="15.5703125" customWidth="1"/>
+    <col min="3" max="9" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="10" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4"/>
     </row>
-    <row r="3" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="76" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="77"/>
-      <c r="C3" s="77"/>
-      <c r="D3" s="77"/>
-      <c r="E3" s="77"/>
-      <c r="F3" s="77"/>
-      <c r="G3" s="77"/>
-      <c r="H3" s="77"/>
-    </row>
-    <row r="4" spans="1:8" ht="30.75" x14ac:dyDescent="0.3">
+      <c r="B3" s="76"/>
+      <c r="C3" s="76"/>
+      <c r="D3" s="76"/>
+      <c r="E3" s="76"/>
+      <c r="F3" s="76"/>
+      <c r="G3" s="76"/>
+      <c r="H3" s="76"/>
+      <c r="I3" s="76"/>
+    </row>
+    <row r="4" spans="1:9" ht="30.75" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
       <c r="F4" s="41" t="s">
         <v>37</v>
@@ -2769,7 +2787,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="C5" s="32"/>
       <c r="D5" s="32"/>
@@ -2786,7 +2804,7 @@
       </c>
       <c r="H5" s="32"/>
     </row>
-    <row r="6" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
       <c r="C6" s="32"/>
       <c r="D6" s="32"/>
@@ -2800,7 +2818,7 @@
       </c>
       <c r="H6" s="32"/>
     </row>
-    <row r="7" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
       <c r="C7" s="32"/>
       <c r="D7" s="32"/>
@@ -2814,7 +2832,7 @@
       </c>
       <c r="H7" s="32"/>
     </row>
-    <row r="8" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="C8" s="32"/>
       <c r="D8" s="32"/>
@@ -2828,7 +2846,7 @@
       </c>
       <c r="H8" s="32"/>
     </row>
-    <row r="9" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
       <c r="C9" s="32"/>
       <c r="D9" s="32"/>
@@ -2842,10 +2860,10 @@
       </c>
       <c r="H9" s="32"/>
     </row>
-    <row r="10" spans="1:8" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
     </row>
-    <row r="11" spans="1:8" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4"/>
       <c r="F11" s="26" t="s">
         <v>64</v>
@@ -2855,25 +2873,26 @@
         <v>#REF!</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4"/>
     </row>
-    <row r="13" spans="1:8" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="79" t="s">
+    <row r="13" spans="1:9" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="82" t="s">
         <v>65</v>
       </c>
-      <c r="B13" s="79"/>
-      <c r="C13" s="79"/>
-      <c r="D13" s="79"/>
-      <c r="E13" s="79"/>
-      <c r="F13" s="79"/>
-      <c r="G13" s="79"/>
-      <c r="H13" s="79"/>
-    </row>
-    <row r="14" spans="1:8" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="82"/>
+      <c r="C13" s="82"/>
+      <c r="D13" s="82"/>
+      <c r="E13" s="82"/>
+      <c r="F13" s="82"/>
+      <c r="G13" s="82"/>
+      <c r="H13" s="82"/>
+      <c r="I13" s="82"/>
+    </row>
+    <row r="14" spans="1:9" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4"/>
     </row>
-    <row r="15" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C15" s="16" t="s">
         <v>57</v>
       </c>
@@ -2889,8 +2908,14 @@
       <c r="G15" s="16" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="H15" s="86" t="s">
+        <v>68</v>
+      </c>
+      <c r="I15" s="86" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="70"/>
       <c r="B16" s="49" t="s">
         <v>16</v>
@@ -2906,13 +2931,21 @@
       <c r="E16" s="25"/>
       <c r="F16" s="25"/>
       <c r="G16" s="25"/>
-    </row>
-    <row r="17" spans="1:8" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H16" s="22">
+        <f t="shared" ref="H16:H21" si="0">G16 -F16</f>
+        <v>0</v>
+      </c>
+      <c r="I16" s="87" t="e">
+        <f t="shared" ref="I16:I21" si="1">H16 /F16</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C17" s="25" t="e">
-        <f t="shared" ref="C17:C21" si="0">G17/(E17*100)</f>
+        <f t="shared" ref="C17:C21" si="2">G17/(E17*100)</f>
         <v>#DIV/0!</v>
       </c>
       <c r="D17" s="25" t="e">
@@ -2922,13 +2955,21 @@
       <c r="E17" s="25"/>
       <c r="F17" s="25"/>
       <c r="G17" s="25"/>
-    </row>
-    <row r="18" spans="1:8" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H17" s="22">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I17" s="87" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="2" t="s">
         <v>5</v>
       </c>
       <c r="C18" s="25" t="e">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="D18" s="25" t="e">
@@ -2938,13 +2979,21 @@
       <c r="E18" s="25"/>
       <c r="F18" s="25"/>
       <c r="G18" s="25"/>
-    </row>
-    <row r="19" spans="1:8" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H18" s="22">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I18" s="87" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="2" t="s">
         <v>6</v>
       </c>
       <c r="C19" s="25" t="e">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="D19" s="25" t="e">
@@ -2954,13 +3003,21 @@
       <c r="E19" s="25"/>
       <c r="F19" s="25"/>
       <c r="G19" s="25"/>
-    </row>
-    <row r="20" spans="1:8" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H19" s="22">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I19" s="87" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C20" s="25" t="e">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="D20" s="25" t="e">
@@ -2970,13 +3027,21 @@
       <c r="E20" s="25"/>
       <c r="F20" s="25"/>
       <c r="G20" s="25"/>
-    </row>
-    <row r="21" spans="1:8" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H20" s="22">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I20" s="87" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="2" t="s">
         <v>39</v>
       </c>
       <c r="C21" s="25" t="e">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>#DIV/0!</v>
       </c>
       <c r="D21" s="25" t="e">
@@ -2986,8 +3051,16 @@
       <c r="E21" s="25"/>
       <c r="F21" s="25"/>
       <c r="G21" s="25"/>
-    </row>
-    <row r="22" spans="1:8" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H21" s="22">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I21" s="87" t="e">
+        <f t="shared" si="1"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="9"/>
       <c r="C22" s="24"/>
       <c r="D22" s="6" t="s">
@@ -3005,24 +3078,29 @@
         <f>SUM(G16:G21)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" s="35" customFormat="1" ht="63" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="78" t="s">
+      <c r="H22" s="24">
+        <f>SUM(H16:H21)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" s="35" customFormat="1" ht="63" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="81" t="s">
         <v>63</v>
       </c>
-      <c r="B24" s="78"/>
-      <c r="C24" s="78"/>
-      <c r="D24" s="78"/>
-      <c r="E24" s="78"/>
-      <c r="F24" s="78"/>
-      <c r="G24" s="78"/>
-      <c r="H24" s="78"/>
+      <c r="B24" s="81"/>
+      <c r="C24" s="81"/>
+      <c r="D24" s="81"/>
+      <c r="E24" s="81"/>
+      <c r="F24" s="81"/>
+      <c r="G24" s="81"/>
+      <c r="H24" s="81"/>
+      <c r="I24" s="81"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A24:H24"/>
-    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A13:I13"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A24:I24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3053,15 +3131,15 @@
       <c r="A3" s="76" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="77"/>
-      <c r="C3" s="77"/>
-      <c r="D3" s="77"/>
-      <c r="E3" s="77"/>
-      <c r="F3" s="77"/>
-      <c r="G3" s="77"/>
-      <c r="H3" s="77"/>
-      <c r="I3" s="77"/>
-      <c r="J3" s="82"/>
+      <c r="B3" s="78"/>
+      <c r="C3" s="78"/>
+      <c r="D3" s="78"/>
+      <c r="E3" s="78"/>
+      <c r="F3" s="78"/>
+      <c r="G3" s="78"/>
+      <c r="H3" s="78"/>
+      <c r="I3" s="78"/>
+      <c r="J3" s="80"/>
     </row>
     <row r="4" spans="1:10" ht="30.75" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
@@ -3598,15 +3676,15 @@
       <c r="A3" s="76" t="s">
         <v>48</v>
       </c>
-      <c r="B3" s="77"/>
-      <c r="C3" s="77"/>
-      <c r="D3" s="77"/>
-      <c r="E3" s="77"/>
-      <c r="F3" s="77"/>
-      <c r="G3" s="77"/>
-      <c r="H3" s="77"/>
-      <c r="I3" s="77"/>
-      <c r="J3" s="82"/>
+      <c r="B3" s="78"/>
+      <c r="C3" s="78"/>
+      <c r="D3" s="78"/>
+      <c r="E3" s="78"/>
+      <c r="F3" s="78"/>
+      <c r="G3" s="78"/>
+      <c r="H3" s="78"/>
+      <c r="I3" s="78"/>
+      <c r="J3" s="80"/>
     </row>
     <row r="4" spans="1:10" ht="41.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>

</xml_diff>